<commit_message>
scan: seg5 2026-10-10 00:11 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-10-08.xlsx
+++ b/output/full_scan/batch_seq6_2026-10-08.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>79.46498954188367</v>
+        <v>79.46498951945375</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>26.3002258251073</v>
+        <v>26.30022595783974</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.294172705056316</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>6.943640669633746</v>
+        <v>6.943640670234652</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
         <v>57.76986786145059</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>14.0018633442272</v>
+        <v>14.00186336069156</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.948459975295852</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.2133900465064079</v>
+        <v>0.2133900464583404</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>69.08680421173534</v>
+        <v>69.08680418374368</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>29.20356209877885</v>
+        <v>29.20356208008065</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>1.04617977215236</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.9124050477091998</v>
+        <v>0.9124050478293766</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>61.76356253115798</v>
+        <v>61.76356252876057</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>14.85445712645613</v>
+        <v>14.85445713839782</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>1.899798463853325</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>6.305596094590224</v>
+        <v>6.305596094830549</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>76.14308286109279</v>
+        <v>76.14308282655526</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>34.31829026227608</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>4.20984272989474</v>
+        <v>4.209842730014904</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>996.0708311342815</v>
+        <v>996.0708311342833</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>674</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>74.85405231427151</v>
+        <v>74.8540523035328</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>35.9147292473659</v>
+        <v>35.91472929688045</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.6242723612538802</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>13.64172907508216</v>
+        <v>13.64172907652414</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>73.37984875248804</v>
+        <v>73.37984875610198</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>25.61489844028412</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>1.950135784910396</v>
+        <v>1.950135784886359</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>81.46445782471895</v>
+        <v>81.46445777236974</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>37.07336608920084</v>
+        <v>37.07336610448105</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>1.64178220010628</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.4529599017441894</v>
+        <v>0.4529599017802407</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>65.24907101546721</v>
+        <v>65.2490707613064</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>19.69315240545272</v>
+        <v>19.69315240784088</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.344300814691493</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.6834629201660084</v>
+        <v>0.6834629202861819</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>68.89639463551066</v>
+        <v>68.89639465361061</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>25.56806467603485</v>
+        <v>25.56806469165961</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.265613054317315</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>30.39538346955518</v>
+        <v>30.39538346919463</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>69.97278570886206</v>
+        <v>69.97278569078239</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>18.45591780997578</v>
+        <v>18.45591782790046</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>4.362155599929602</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>6.89737592200013</v>
+        <v>6.897375923322028</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>75.33749264635546</v>
+        <v>75.33749259721402</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>26.50443267888965</v>
+        <v>26.50443270267381</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.565433896382268</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.2096643150977287</v>
+        <v>0.2096643151337769</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1191,7 +1191,7 @@
         <v>72.62807070791342</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>34.35690854750507</v>
+        <v>34.35690855663209</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.471073908331133</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>4.250877640073545</v>
+        <v>4.250877639953369</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1227,7 +1227,7 @@
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>885.7592487529702</v>
+        <v>885.7592487529703</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1740</v>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>67.59519846659254</v>
+        <v>67.59519842116066</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>24.52050905404415</v>
+        <v>24.52050901694153</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.8230606874435739</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>36.04697196251469</v>
+        <v>36.04697197008559</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>59.88611552561413</v>
+        <v>59.88611554884109</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>16.82826803470885</v>
+        <v>16.82826798296572</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.901939468960706</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.3115398574404739</v>
+        <v>0.3115398573563533</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>64.0805765719719</v>
+        <v>64.08057648556726</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>20.23027685021475</v>
+        <v>20.23027684660553</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>1.279024845270974</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.0999853223530497</v>
+        <v>0.0999853224972547</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>838.2033652565141</v>
+        <v>838.2033652565192</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>76.5</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>67.17796667224516</v>
+        <v>67.17796653183512</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>23.15136196679104</v>
+        <v>23.15136200008063</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.058643954916541</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.9227012507353138</v>
+        <v>0.9227012515044336</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>55.43677585189899</v>
+        <v>55.43677589650424</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>32.04125259484862</v>
+        <v>32.04125263799971</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.3205447993659142</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.2588872808783855</v>
+        <v>0.2588872806260247</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>67.80021508070274</v>
+        <v>67.80021503842451</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>35.84827103040959</v>
+        <v>35.84827095327165</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.363261771975065</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.9794340003327732</v>
+        <v>0.9794340006452172</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>68.1964983983091</v>
+        <v>68.19649827556573</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>26.39994667318064</v>
+        <v>26.39994673087083</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.7283742089832541</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-1.068668999753154</v>
+        <v>-1.068668999512821</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>776.9056086942354</v>
+        <v>776.9056086942352</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>88</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>57.55349529316179</v>
+        <v>57.55349522059731</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>32.3992546215789</v>
+        <v>32.39925462320264</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.4282643300109952</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.1197724852938846</v>
+        <v>0.11977248541407</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>64.43952001476103</v>
+        <v>64.43951999707458</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>20.54028035680201</v>
+        <v>20.54028037329116</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.7635946244863818</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>3.549193878831565</v>
+        <v>3.549193878230716</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>776.1255125146679</v>
+        <v>776.1255125146681</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>308</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>61.54013601219298</v>
+        <v>61.54013598821194</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>18.26157809998703</v>
+        <v>18.2615780754512</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>1.06746148933019</v>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>64.13753878107569</v>
+        <v>64.13753879383111</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>31.22081947259757</v>
+        <v>31.22081972788407</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.7072389501012587</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.6257119065077337</v>
+        <v>0.6257119062914382</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>60.81933929535338</v>
+        <v>60.81933930311666</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>34.49426503798122</v>
+        <v>34.49426505452639</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>0.8989905060510612</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>62.60319953987802</v>
+        <v>62.60319950201166</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>21.19958399299881</v>
+        <v>21.19958398773892</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.491185109352189</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1.184233753019253</v>
+        <v>1.184233752899068</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>66.88591428927262</v>
+        <v>66.88591420944987</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>25.47116182379192</v>
+        <v>25.47116182928336</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>2.654281188155089</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>2.30008796049709</v>
+        <v>2.300087960857613</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>726.3653569529293</v>
+        <v>726.3653569529291</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>164.5</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>64.1045871838121</v>
+        <v>64.10458709152351</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>33.00391610482491</v>
+        <v>33.0039160886967</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.5731948857269488</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>73.60107202132252</v>
+        <v>73.60107203857173</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>38.96617212676106</v>
+        <v>38.96617216672738</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.050323715575384</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2.589627552312971</v>
+        <v>2.589627552385074</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>65.36613798976518</v>
+        <v>65.3661380445343</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>20.33079371275281</v>
+        <v>20.330793728338</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.967500366775817</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>0.503035591230281</v>
+        <v>0.5030355912062466</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>63.64952481305248</v>
+        <v>63.64952478840734</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>23.43117289222213</v>
+        <v>23.43117289688426</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.6748206494924659</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>0.7641007326486333</v>
+        <v>0.7641007326967051</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>60.6903955107796</v>
+        <v>60.69039550604356</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>43.02121234288609</v>
+        <v>43.0212122671155</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.3196013781485974</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3486736116813951</v>
+        <v>0.3486736117054549</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>55.98040445119885</v>
+        <v>55.98040444462473</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>52.14993814183419</v>
+        <v>52.14993800182121</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.7053283181476214</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.3481175606845363</v>
+        <v>-0.3481175606965543</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>64.76383459061591</v>
+        <v>64.76383463160613</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>34.2082555775107</v>
+        <v>34.20825560185507</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.3660689049433483</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>2.391347895237356</v>
+        <v>2.391347895333508</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>61.69089634572368</v>
+        <v>61.69089634130896</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>49.45772430235029</v>
+        <v>49.45772446632229</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.9719224449878356</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.5618640143941773</v>
+        <v>-0.561864014370137</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>52.71695150247466</v>
+        <v>52.71695156270656</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>20.013255353472</v>
+        <v>20.01325549556053</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1.402185711225031</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>1.186821073077724</v>
+        <v>1.186821072356692</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2446,7 +2446,7 @@
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>643.8982457148588</v>
+        <v>643.8982457148592</v>
       </c>
       <c r="E38" s="2" t="n">
         <v>1785</v>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>61.46122239330042</v>
+        <v>61.46122231276667</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>19.96090391438413</v>
+        <v>19.9609038693042</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>1.60955027857943</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>25.75823223680413</v>
+        <v>25.75823224954256</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>52.38817048253696</v>
+        <v>52.38817044820993</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>35.0887059228752</v>
+        <v>35.0887055714697</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.73081792615375</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.0593069296777939</v>
+        <v>-0.0593069295095383</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>68.06947570820074</v>
+        <v>68.06947568963692</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>18.25948553084111</v>
+        <v>18.25948552114786</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.4558432423076169</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.1854615388077896</v>
+        <v>0.185461538783755</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>627.7461519627847</v>
+        <v>627.7461519627835</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>49.3</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>55.20855805694176</v>
+        <v>55.20855832864774</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>22.76966617056219</v>
+        <v>22.76966613917228</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.3847961847088648</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>0.1091770830115376</v>
+        <v>0.1091770824827835</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.30982307928421</v>
+        <v>52.30982307022713</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>43.59201869689436</v>
+        <v>43.59201887965735</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>1.057899367362755</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.9911700939335608</v>
+        <v>-0.9911700938374252</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>54.30925141236648</v>
+        <v>54.30925154084466</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>18.41900796797728</v>
+        <v>18.41900799872784</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.8109504080699972</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>3.678470891736591</v>
+        <v>3.67847089053484</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>51.81417153388654</v>
+        <v>51.81417152994361</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>38.46113765395066</v>
+        <v>38.46113759337639</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.2894454963500344</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-4.75790448925655</v>
+        <v>-4.757904489102373</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>55.63742710638107</v>
+        <v>55.63742709707654</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>35.45056269081356</v>
+        <v>35.45056275432712</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>1.884320724978657</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>0.2191252318443066</v>
+        <v>0.2191252318803594</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>57.48413967295054</v>
+        <v>57.48413961307436</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>32.60549729179129</v>
+        <v>32.60549737115372</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.4592541442673478</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>-0.120355735333824</v>
+        <v>-0.1203557348531561</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>57.47913295397071</v>
+        <v>57.4791329512662</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>25.99878212565197</v>
+        <v>25.99878213888796</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.8229034555679852</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>1.384159071161655</v>
+        <v>1.384159071185698</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>58.64477782510787</v>
+        <v>58.64477781140761</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>32.24959475455059</v>
+        <v>32.24959476416474</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.5174583600909997</v>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>50.29496227308474</v>
+        <v>50.29496219029219</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>26.60156292041889</v>
+        <v>26.60156294589656</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.8015324316162563</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.7327123175847614</v>
+        <v>0.7327123180414186</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>48.91182294386238</v>
+        <v>48.91182300432327</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>29.91343594332426</v>
+        <v>29.91343593099582</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.3820741227775743</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-1.183048540124158</v>
+        <v>-1.183048540028014</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>54.67810206496629</v>
+        <v>54.67810206222514</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>37.75453483422483</v>
+        <v>37.75453484699413</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.7857190156112829</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-6.176283630135124</v>
+        <v>-6.176283630183171</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>54.92194317442267</v>
+        <v>54.92194303358973</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>35.1029317777166</v>
+        <v>35.10293177771661</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.9567766258121844</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.0958878190139032</v>
+        <v>0.0958878192061835</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>56.53207817580785</v>
+        <v>56.53207818867043</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>25.56686262549697</v>
+        <v>25.56686271197566</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.6293160744192784</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>1.146203546143385</v>
+        <v>1.146203546083294</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>496.6894975653068</v>
+        <v>496.6894975653069</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>1195</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>45.1647860360041</v>
+        <v>45.16478603228927</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>15.34007685143156</v>
+        <v>15.3400768836689</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.6169973544641724</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>4.977192496395062</v>
+        <v>4.977192495673904</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>490.5561638857645</v>
+        <v>490.556163885765</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>87.7</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>54.27043194283701</v>
+        <v>54.27043196744194</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>25.42311787074285</v>
+        <v>25.42311788262887</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.5829207772436857</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0393786941462823</v>
+        <v>0.0393786939540063</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>486.5628000316162</v>
+        <v>486.5628000316183</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>115.5</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>57.79831896721706</v>
+        <v>57.79831864149693</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>18.79603346803991</v>
+        <v>18.79603350054156</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.3880258780331017</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.484835822651646</v>
+        <v>0.4848358238533723</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>473.33627582486</v>
+        <v>473.3362758248573</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>24.1</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>56.67365361416208</v>
+        <v>56.67365356137509</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>19.9889933015307</v>
+        <v>19.98899331611396</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>0.6706224607875299</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0498264658311689</v>
+        <v>0.0498264658672204</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>472.9037658122512</v>
+        <v>472.9037658122501</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>5575</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>52.04528800116154</v>
+        <v>52.04528798519506</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>11.69305823744509</v>
+        <v>11.69305830808589</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.5728205667649403</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>31.46568161468948</v>
+        <v>31.46568161829496</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>468.0328157905217</v>
+        <v>468.0328157905218</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>421</v>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>49.67736785338496</v>
+        <v>49.67736786122421</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>28.835958292447</v>
+        <v>28.83595829267376</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>0.6471612400226758</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.0550277861415358</v>
+        <v>-0.0550277873432746</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>50.87352637436982</v>
+        <v>50.87352638483091</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>17.92504452498463</v>
+        <v>17.92504458256967</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.163762772921273</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.3501849271105745</v>
+        <v>0.3501849270504911</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.1032947298192</v>
+        <v>50.10329477465732</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>21.55546829569838</v>
+        <v>21.55546833489858</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.4259700814411203</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1056811239041529</v>
+        <v>0.1056811238801204</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>448.5378324189813</v>
+        <v>448.5378324189812</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>100.5</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>48.32285828637959</v>
+        <v>48.32285850939702</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>20.040948937815</v>
+        <v>20.0409489217368</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3640116687412575</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>0.1629282914240892</v>
+        <v>0.1629282895013101</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,7 +3785,7 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>51.00808673813849</v>
+        <v>51.00808682562293</v>
       </c>
       <c r="I63" s="2" t="n">
         <v>29.57421617637868</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.8889113862040228</v>
+        <v>0.8889113857233217</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>42.38974280327943</v>
+        <v>42.38974276410438</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.7359633916341</v>
+        <v>16.73596341283164</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.1674061600921483</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.3328560194458895</v>
+        <v>-0.3328560194699223</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>439.4613797171348</v>
+        <v>439.4613797171333</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>39.5</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>54.70594203827836</v>
+        <v>54.70594195388935</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>24.35656301897063</v>
+        <v>24.35656326934681</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>2.407765344398479</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.2280600990058658</v>
+        <v>0.2280600992101636</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.84522978981229</v>
+        <v>47.84522980760068</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>7.540572312280814</v>
+        <v>7.540572314720303</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.5769033129826593</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.8792172338603175</v>
+        <v>0.8792172326586023</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>45.0849308053389</v>
+        <v>45.08493081167318</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>16.63049652299429</v>
+        <v>16.63049660300517</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4978613986623879</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.2562077696609277</v>
+        <v>0.2562077696489016</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4036,7 +4036,7 @@
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>407.9725395491897</v>
+        <v>407.9725395491898</v>
       </c>
       <c r="E68" s="2" t="n">
         <v>103.5</v>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>46.61624856703296</v>
+        <v>46.61624858052419</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>32.72428098669584</v>
+        <v>32.72428100571619</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>1.690507786029236</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.604376876693282</v>
+        <v>0.6043768766211819</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>51.93485825291294</v>
+        <v>51.93485826412152</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>3.521058822162868</v>
+        <v>3.52105891112504</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>1.140350288776941</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0643474599042566</v>
+        <v>0.0643474598922385</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>47.84633261046508</v>
+        <v>47.84633247749867</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>27.87336314441082</v>
+        <v>27.87336329965351</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.7365897181654893</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.3077326702286176</v>
+        <v>0.3077326707093224</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>400.3228159019485</v>
+        <v>400.3228159019436</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>27</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>50.96708635200682</v>
+        <v>50.96708633877626</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>28.9935678727525</v>
+        <v>28.99356786898994</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.3424332478416957</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.134839972081054</v>
+        <v>0.134839972117105</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>42.22283952548904</v>
+        <v>42.22283951459619</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>23.78749696023577</v>
+        <v>23.78749700255358</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.9376283161202454</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-8.477996267734937</v>
+        <v>-8.477996268816465</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4301,7 +4301,7 @@
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>386.5852268132572</v>
+        <v>386.5852268132571</v>
       </c>
       <c r="E73" s="2" t="n">
         <v>18</v>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>55.29037478876737</v>
+        <v>55.29037482554875</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>14.52618586262748</v>
+        <v>14.52618580699394</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>2.70414668793422</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.8087945813965822</v>
+        <v>0.8087945811322008</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>382.0103818425441</v>
+        <v>382.0103818425447</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>43.2</v>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>45.18083497098547</v>
+        <v>45.18083497580241</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>15.417570663253</v>
+        <v>15.41757064844356</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.088988554589016</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.2400524017806486</v>
+        <v>0.2400524016003936</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>42.30951235131371</v>
+        <v>42.30951237502908</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>13.91767579666506</v>
+        <v>13.91767587455112</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.7527343987928723</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.6734510059318398</v>
+        <v>-0.6734510062923745</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>44.12994973743514</v>
+        <v>44.12994948286578</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>20.05400858504866</v>
+        <v>20.05400860442172</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>2.921391987367654</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0208119116676522</v>
+        <v>-0.0208119113311681</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>358.4760665744067</v>
+        <v>358.4760665744066</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>78.90000000000001</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>52.67415913903354</v>
+        <v>52.67415914763877</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>16.76882189620423</v>
+        <v>16.76882190490386</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.6159773522481475</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.5296212085930062</v>
+        <v>0.5296212084488022</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>44.78915607188766</v>
+        <v>44.78915594431876</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>14.37777899772824</v>
+        <v>14.37777906156054</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.2960801209436421</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.1373280435295672</v>
+        <v>-0.1373280434334248</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>51.57313431378976</v>
+        <v>51.5731342558962</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>18.10069650631083</v>
+        <v>18.10069645620608</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.8006348097026877</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.7544665883053154</v>
+        <v>0.7544665881851427</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4689,7 +4689,7 @@
         <v>38.38011919470132</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>19.31500520721642</v>
+        <v>19.31500566654826</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>1.835561939772701</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.0242238456906397</v>
+        <v>0.0242238457507254</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>52.60938929429401</v>
+        <v>52.6093892832286</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>16.62940385459855</v>
+        <v>16.62940393602072</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.4874922537721792</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>2.126052321378357</v>
+        <v>2.126052321162021</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>40.74956787591968</v>
+        <v>40.74956787711988</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>15.30262190307135</v>
+        <v>15.30262193866628</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-1.827411258314468</v>
+        <v>-1.827411258146226</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>47.47659813469829</v>
+        <v>47.47659796923825</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>15.00981422852612</v>
+        <v>15.00981420792055</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.8604789287030653</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.1101373656368981</v>
+        <v>0.1101373657090015</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>323.5126855444195</v>
+        <v>323.5126855444196</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>34.3</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>49.66622949997304</v>
+        <v>49.66622880371294</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>31.5832025205298</v>
+        <v>31.58320256157418</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.6850230461123523</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.145748121689812</v>
+        <v>-0.1457481210168421</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>48.77258409237539</v>
+        <v>48.77258351304166</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>14.02569976876042</v>
+        <v>14.02569956253096</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.9922289282288724</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0238215498603316</v>
+        <v>0.0238215499564229</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>41.64580686829242</v>
+        <v>41.64580683957967</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>9.406252666683258</v>
+        <v>9.406252627375869</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>1.185098328064244</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.1797636419483321</v>
+        <v>0.1797636418865478</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>318.7914421473522</v>
+        <v>318.7914421473526</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>62.5</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>41.61559882823463</v>
+        <v>41.61559746803179</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>24.89577662866258</v>
+        <v>24.89577718367942</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.205240586704962</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>0.325304199880271</v>
+        <v>0.3253042019232228</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>317.339954911232</v>
+        <v>317.3399549112315</v>
       </c>
       <c r="E88" s="2" t="n">
         <v>168</v>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>46.34067468086418</v>
+        <v>46.34067470833464</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>13.64863592572729</v>
+        <v>13.64863608443968</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.8816950788172239</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.1069853220640617</v>
+        <v>-0.106985322280404</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>44.55516494287926</v>
+        <v>44.55516487384117</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>7.741277903514341</v>
+        <v>7.741277907761123</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.061630723977469</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>41.10006100095028</v>
+        <v>41.10006108390709</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>14.25526461937799</v>
+        <v>14.25526465804545</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.523325087508403</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.09937463424993841</v>
+        <v>0.099374634273968</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>299.9093986416535</v>
+        <v>299.9093986416524</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>36.1</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>33.25295697484269</v>
+        <v>33.25295701424386</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.40203552758541</v>
+        <v>16.40203578324442</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>1.636353862264569</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.2409906207560992</v>
+        <v>-0.2409906211406553</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>48.77287710712907</v>
+        <v>48.77287693644514</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.51442681894661</v>
+        <v>12.51442687779584</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.4348668324621864</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.2541926796307566</v>
+        <v>-0.2541926800426635</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>291.317210347153</v>
+        <v>291.3172103471529</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>59.9</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>46.17215873510872</v>
+        <v>46.17215950310087</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>9.216922855944976</v>
+        <v>9.216922880374089</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>1.249264594028412</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.09504237893361581</v>
+        <v>0.0950423781885453</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>45.11486981408318</v>
+        <v>45.11486982112562</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>14.47422050402955</v>
+        <v>14.47422045229279</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.3811414374332916</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.2262497860322402</v>
+        <v>0.2262497860442558</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>41.76788306841641</v>
+        <v>41.76788383077785</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>25.9540047359469</v>
+        <v>25.95400442126441</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.2089990252039252</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.0533109120463983</v>
+        <v>0.0533109114936002</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>51.488743295798</v>
+        <v>51.48874331515211</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>7.413113537644509</v>
+        <v>7.413113448963617</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.0616895534910118</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.2830577764091596</v>
+        <v>0.2830577763731065</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>274.1807817869298</v>
+        <v>274.1807817869297</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>25.8</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>48.05776732579494</v>
+        <v>48.05776733780432</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>20.95541984737102</v>
+        <v>20.95541979695023</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4051523792768494</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>45.07401217972424</v>
+        <v>45.07401198473636</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>12.06075918347341</v>
+        <v>12.06075913841485</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.6677909634672433</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.1392495284820216</v>
+        <v>-0.1392495279532573</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.69041987627492</v>
+        <v>41.69041962069908</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.73243016912364</v>
+        <v>16.73243041459309</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4163025262967711</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0685617920240111</v>
+        <v>0.0685617919278729</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>255.0471086599354</v>
+        <v>255.0471086599353</v>
       </c>
       <c r="E100" s="2" t="n">
         <v>93.3</v>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>36.11295329110976</v>
+        <v>36.11295278503218</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>9.798471226473838</v>
+        <v>9.798471254467136</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>2.487407043997548</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.1935775210738975</v>
+        <v>-0.193577520112533</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>44.62086216214763</v>
+        <v>44.62086219667224</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>22.76719014609892</v>
+        <v>22.76719004007565</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.0758739211042115</v>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>238.3841345843215</v>
+        <v>238.3841345843227</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>22.3</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>40.93586023042185</v>
+        <v>40.93586028822313</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.03011852028452</v>
+        <v>17.03011854407021</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.9075224382208136</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0419286807018686</v>
+        <v>-0.0419286807138878</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>231.0569135764281</v>
+        <v>231.056913576428</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>44.15</v>
@@ -5908,7 +5908,7 @@
         <v>43.2078597571998</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>26.98343145902366</v>
+        <v>26.98343172648024</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5685829799822503</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0166069864173007</v>
+        <v>-0.0166069864894063</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>230.3960435151252</v>
+        <v>230.3960435151257</v>
       </c>
       <c r="E104" s="2" t="n">
         <v>51</v>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>47.00197673440443</v>
+        <v>47.00197664977547</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>10.07706021861419</v>
+        <v>10.07706028723438</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.38745756334259</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.0002543061124941</v>
+        <v>-0.0002543060884649</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>228.8653854294278</v>
+        <v>228.8653854294277</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>868</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>37.84148844451587</v>
+        <v>37.84148837808175</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>13.41429763359527</v>
+        <v>13.41429769405833</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.8474657377354361</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>2.889963616940307</v>
+        <v>2.889963613335127</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>227.5962448273092</v>
+        <v>227.596244827311</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>34.65</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>46.662072382813</v>
+        <v>46.66207208234515</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>24.80677598090175</v>
+        <v>24.80677599942341</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.6476808746442609</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0082952622779786</v>
+        <v>-0.008295261809307</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>46.47012988963206</v>
+        <v>46.47012986403792</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>9.076027381227568</v>
+        <v>9.076027414832756</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.3064093180084713</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.0370086347024067</v>
+        <v>0.0370086347144194</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>208.4147303012684</v>
+        <v>208.4147303012683</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>45.95</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>43.44224238305644</v>
+        <v>43.44224236614954</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>12.80225797012829</v>
+        <v>12.80225798746838</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.354691712174793</v>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>192.4196536978067</v>
+        <v>192.4196536978065</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>73</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>32.07702986363576</v>
+        <v>32.07702994424456</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>18.34389015746456</v>
+        <v>18.34388997749882</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>1.450007571509841</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.130055043177476</v>
+        <v>0.1300550426967679</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>42.35688527511441</v>
+        <v>42.35688529633865</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>10.2330487939857</v>
+        <v>10.233048762671</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.958165478506654</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.0012777892768378</v>
+        <v>0.0012777891326254</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>50.52613751987526</v>
+        <v>50.52613753742693</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>16.30507301775355</v>
+        <v>16.30507279431471</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.2102735870154775</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0595770887652129</v>
+        <v>0.0595770885008314</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>148.605901010752</v>
+        <v>148.6059010107519</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>42.75</v>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>48.96324100123464</v>
+        <v>48.96324073018989</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>19.23222113048167</v>
+        <v>19.23222110587582</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.7730287448142529</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0069697375357186</v>
+        <v>0.0069697374876498</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>47.91922590086912</v>
+        <v>47.91922551134112</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>8.780249822181149</v>
+        <v>8.780249705362722</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.963897398420272</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0452194382076676</v>
+        <v>0.0452194386643302</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,7 +6488,7 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.78275577003692</v>
+        <v>45.7827557655602</v>
       </c>
       <c r="I114" s="2" t="n">
         <v>18.70922704152799</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.2373580357377152</v>
+        <v>-0.2373580357016701</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>44.7037802253525</v>
+        <v>44.70378022383345</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>8.288036179015641</v>
+        <v>8.288036290790041</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.0008963585434173</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.6926433050163903</v>
+        <v>-0.692643304968322</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>

</xml_diff>